<commit_message>
Precios EE. UU.: envío nacional más realista (USPS Ground Advantage menos de 1 lb)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp6cWLHDTqXsEaejCBC2fh
</commit_message>
<xml_diff>
--- a/us-filter-store/precios/precios-de-venta.xlsx
+++ b/us-filter-store/precios/precios-de-venta.xlsx
@@ -61,12 +61,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
+        <fgColor rgb="00FDE2E2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDE2E2"/>
+        <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -612,7 +612,7 @@
       </c>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="3" t="n">
-        <v>34.99</v>
+        <v>36.99</v>
       </c>
       <c r="K2" s="2">
         <f>J2-J2*Supuestos!$B$2-Supuestos!$B$3-F2</f>
@@ -683,7 +683,7 @@
       </c>
       <c r="I3" s="2" t="n"/>
       <c r="J3" s="3" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="K3" s="2">
         <f>J3-J3*Supuestos!$B$2-Supuestos!$B$3-F3</f>
@@ -755,28 +755,14 @@
       <c r="I4" s="2" t="n">
         <v>34.99</v>
       </c>
-      <c r="J4" s="3" t="n">
-        <v>37.99</v>
-      </c>
-      <c r="K4" s="2">
-        <f>J4-J4*Supuestos!$B$2-Supuestos!$B$3-F4</f>
-        <v/>
-      </c>
-      <c r="L4" s="4">
-        <f>K4/J4</f>
-        <v/>
-      </c>
-      <c r="M4" s="2">
-        <f>ROUNDUP(MAX(2*J4*0.92,(2*E4+Supuestos!$B$6+Supuestos!$B$3+8)/(1-Supuestos!$B$2)),0)-0.01</f>
-        <v/>
-      </c>
-      <c r="N4" s="2">
-        <f>M4-M4*Supuestos!$B$2-Supuestos!$B$3-2*E4-Supuestos!$B$6</f>
-        <v/>
-      </c>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="4" t="n"/>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>Ganancia justa: igualar al mercado</t>
+          <t>No vender suelto: el mercado está casi al precio de costo</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -832,28 +818,14 @@
       <c r="I5" s="2" t="n">
         <v>36.99</v>
       </c>
-      <c r="J5" s="3" t="n">
-        <v>39.99</v>
-      </c>
-      <c r="K5" s="2">
-        <f>J5-J5*Supuestos!$B$2-Supuestos!$B$3-F5</f>
-        <v/>
-      </c>
-      <c r="L5" s="4">
-        <f>K5/J5</f>
-        <v/>
-      </c>
-      <c r="M5" s="2">
-        <f>ROUNDUP(MAX(2*J5*0.92,(2*E5+Supuestos!$B$6+Supuestos!$B$3+8)/(1-Supuestos!$B$2)),0)-0.01</f>
-        <v/>
-      </c>
-      <c r="N5" s="2">
-        <f>M5-M5*Supuestos!$B$2-Supuestos!$B$3-2*E5-Supuestos!$B$6</f>
-        <v/>
-      </c>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="n"/>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>Ganancia justa: igualar al mercado</t>
+          <t>No vender suelto: el mercado está casi al precio de costo</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -914,7 +886,7 @@
       <c r="L6" s="4" t="n"/>
       <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="n"/>
-      <c r="O6" s="6" t="inlineStr">
+      <c r="O6" s="5" t="inlineStr">
         <is>
           <t>No vender suelto: el mercado está casi al precio de costo</t>
         </is>
@@ -973,7 +945,7 @@
         <v>54.99</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>58.99</v>
+        <v>61.99</v>
       </c>
       <c r="K7" s="2">
         <f>J7-J7*Supuestos!$B$2-Supuestos!$B$3-F7</f>
@@ -1050,7 +1022,7 @@
         <v>54.97</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>56.99</v>
+        <v>59.99</v>
       </c>
       <c r="K8" s="2">
         <f>J8-J8*Supuestos!$B$2-Supuestos!$B$3-F8</f>
@@ -1127,7 +1099,7 @@
         <v>49.99</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>52.99</v>
+        <v>54.99</v>
       </c>
       <c r="K9" s="2">
         <f>J9-J9*Supuestos!$B$2-Supuestos!$B$3-F9</f>
@@ -1145,7 +1117,7 @@
         <f>M9-M9*Supuestos!$B$2-Supuestos!$B$3-2*E9-Supuestos!$B$6</f>
         <v/>
       </c>
-      <c r="O9" s="5" t="inlineStr">
+      <c r="O9" s="6" t="inlineStr">
         <is>
           <t>Ganancia justa: igualar al mercado</t>
         </is>
@@ -1198,7 +1170,7 @@
       </c>
       <c r="I10" s="2" t="n"/>
       <c r="J10" s="3" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="K10" s="2">
         <f>J10-J10*Supuestos!$B$2-Supuestos!$B$3-F10</f>
@@ -1273,7 +1245,7 @@
       </c>
       <c r="I11" s="2" t="n"/>
       <c r="J11" s="3" t="n">
-        <v>56.99</v>
+        <v>59.99</v>
       </c>
       <c r="K11" s="2">
         <f>J11-J11*Supuestos!$B$2-Supuestos!$B$3-F11</f>
@@ -1346,7 +1318,7 @@
         <v>54.99</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>53.99</v>
+        <v>55.99</v>
       </c>
       <c r="K12" s="2">
         <f>J12-J12*Supuestos!$B$2-Supuestos!$B$3-F12</f>
@@ -1421,7 +1393,7 @@
       </c>
       <c r="I13" s="2" t="n"/>
       <c r="J13" s="3" t="n">
-        <v>23.99</v>
+        <v>25.99</v>
       </c>
       <c r="K13" s="2">
         <f>J13-J13*Supuestos!$B$2-Supuestos!$B$3-F13</f>
@@ -1488,7 +1460,7 @@
       </c>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="3" t="n">
-        <v>33.99</v>
+        <v>35.99</v>
       </c>
       <c r="K14" s="2">
         <f>J14-J14*Supuestos!$B$2-Supuestos!$B$3-F14</f>
@@ -1565,7 +1537,7 @@
       <c r="L15" s="4" t="n"/>
       <c r="M15" s="2" t="n"/>
       <c r="N15" s="2" t="n"/>
-      <c r="O15" s="6" t="inlineStr">
+      <c r="O15" s="5" t="inlineStr">
         <is>
           <t>No vender suelto: el mercado está casi al precio de costo</t>
         </is>
@@ -1618,7 +1590,7 @@
       </c>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="3" t="n">
-        <v>65.98999999999999</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="K16" s="2">
         <f>J16-J16*Supuestos!$B$2-Supuestos!$B$3-F16</f>
@@ -1693,7 +1665,7 @@
       </c>
       <c r="I17" s="2" t="n"/>
       <c r="J17" s="3" t="n">
-        <v>65.98999999999999</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="K17" s="2">
         <f>J17-J17*Supuestos!$B$2-Supuestos!$B$3-F17</f>
@@ -1760,7 +1732,7 @@
       </c>
       <c r="I18" s="2" t="n"/>
       <c r="J18" s="3" t="n">
-        <v>53.99</v>
+        <v>55.99</v>
       </c>
       <c r="K18" s="2">
         <f>J18-J18*Supuestos!$B$2-Supuestos!$B$3-F18</f>
@@ -1827,7 +1799,7 @@
       </c>
       <c r="I19" s="2" t="n"/>
       <c r="J19" s="3" t="n">
-        <v>113.99</v>
+        <v>116.99</v>
       </c>
       <c r="K19" s="2">
         <f>J19-J19*Supuestos!$B$2-Supuestos!$B$3-F19</f>
@@ -1894,7 +1866,7 @@
       </c>
       <c r="I20" s="2" t="n"/>
       <c r="J20" s="3" t="n">
-        <v>56.99</v>
+        <v>58.99</v>
       </c>
       <c r="K20" s="2">
         <f>J20-J20*Supuestos!$B$2-Supuestos!$B$3-F20</f>
@@ -1961,7 +1933,7 @@
       </c>
       <c r="I21" s="2" t="n"/>
       <c r="J21" s="3" t="n">
-        <v>87.98999999999999</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="K21" s="2">
         <f>J21-J21*Supuestos!$B$2-Supuestos!$B$3-F21</f>
@@ -2028,7 +2000,7 @@
       </c>
       <c r="I22" s="2" t="n"/>
       <c r="J22" s="3" t="n">
-        <v>90.98999999999999</v>
+        <v>92.98999999999999</v>
       </c>
       <c r="K22" s="2">
         <f>J22-J22*Supuestos!$B$2-Supuestos!$B$3-F22</f>
@@ -2095,7 +2067,7 @@
       </c>
       <c r="I23" s="2" t="n"/>
       <c r="J23" s="3" t="n">
-        <v>66.98999999999999</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="K23" s="2">
         <f>J23-J23*Supuestos!$B$2-Supuestos!$B$3-F23</f>
@@ -2162,7 +2134,7 @@
       </c>
       <c r="I24" s="2" t="n"/>
       <c r="J24" s="3" t="n">
-        <v>89.98999999999999</v>
+        <v>91.98999999999999</v>
       </c>
       <c r="K24" s="2">
         <f>J24-J24*Supuestos!$B$2-Supuestos!$B$3-F24</f>
@@ -2229,7 +2201,7 @@
       </c>
       <c r="I25" s="2" t="n"/>
       <c r="J25" s="3" t="n">
-        <v>49.99</v>
+        <v>51.99</v>
       </c>
       <c r="K25" s="2">
         <f>J25-J25*Supuestos!$B$2-Supuestos!$B$3-F25</f>
@@ -2296,7 +2268,7 @@
       </c>
       <c r="I26" s="2" t="n"/>
       <c r="J26" s="3" t="n">
-        <v>89.98999999999999</v>
+        <v>91.98999999999999</v>
       </c>
       <c r="K26" s="2">
         <f>J26-J26*Supuestos!$B$2-Supuestos!$B$3-F26</f>
@@ -2363,7 +2335,7 @@
       </c>
       <c r="I27" s="2" t="n"/>
       <c r="J27" s="3" t="n">
-        <v>35.99</v>
+        <v>37.99</v>
       </c>
       <c r="K27" s="2">
         <f>J27-J27*Supuestos!$B$2-Supuestos!$B$3-F27</f>
@@ -2430,7 +2402,7 @@
       </c>
       <c r="I28" s="2" t="n"/>
       <c r="J28" s="3" t="n">
-        <v>52.99</v>
+        <v>54.99</v>
       </c>
       <c r="K28" s="2">
         <f>J28-J28*Supuestos!$B$2-Supuestos!$B$3-F28</f>
@@ -2497,7 +2469,7 @@
       </c>
       <c r="I29" s="2" t="n"/>
       <c r="J29" s="3" t="n">
-        <v>50.99</v>
+        <v>53.99</v>
       </c>
       <c r="K29" s="2">
         <f>J29-J29*Supuestos!$B$2-Supuestos!$B$3-F29</f>
@@ -2564,7 +2536,7 @@
       </c>
       <c r="I30" s="2" t="n"/>
       <c r="J30" s="3" t="n">
-        <v>27.99</v>
+        <v>30.99</v>
       </c>
       <c r="K30" s="2">
         <f>J30-J30*Supuestos!$B$2-Supuestos!$B$3-F30</f>
@@ -2631,7 +2603,7 @@
       </c>
       <c r="I31" s="2" t="n"/>
       <c r="J31" s="3" t="n">
-        <v>37.99</v>
+        <v>39.99</v>
       </c>
       <c r="K31" s="2">
         <f>J31-J31*Supuestos!$B$2-Supuestos!$B$3-F31</f>
@@ -2698,7 +2670,7 @@
       </c>
       <c r="I32" s="2" t="n"/>
       <c r="J32" s="3" t="n">
-        <v>29.99</v>
+        <v>31.99</v>
       </c>
       <c r="K32" s="2">
         <f>J32-J32*Supuestos!$B$2-Supuestos!$B$3-F32</f>
@@ -2765,7 +2737,7 @@
       </c>
       <c r="I33" s="2" t="n"/>
       <c r="J33" s="3" t="n">
-        <v>61.99</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="K33" s="2">
         <f>J33-J33*Supuestos!$B$2-Supuestos!$B$3-F33</f>
@@ -2832,7 +2804,7 @@
       </c>
       <c r="I34" s="2" t="n"/>
       <c r="J34" s="3" t="n">
-        <v>30.99</v>
+        <v>32.99</v>
       </c>
       <c r="K34" s="2">
         <f>J34-J34*Supuestos!$B$2-Supuestos!$B$3-F34</f>
@@ -2899,7 +2871,7 @@
       </c>
       <c r="I35" s="2" t="n"/>
       <c r="J35" s="3" t="n">
-        <v>36.99</v>
+        <v>38.99</v>
       </c>
       <c r="K35" s="2">
         <f>J35-J35*Supuestos!$B$2-Supuestos!$B$3-F35</f>
@@ -2966,7 +2938,7 @@
       </c>
       <c r="I36" s="2" t="n"/>
       <c r="J36" s="3" t="n">
-        <v>59.99</v>
+        <v>62.99</v>
       </c>
       <c r="K36" s="2">
         <f>J36-J36*Supuestos!$B$2-Supuestos!$B$3-F36</f>
@@ -3033,7 +3005,7 @@
       </c>
       <c r="I37" s="2" t="n"/>
       <c r="J37" s="3" t="n">
-        <v>56.99</v>
+        <v>59.99</v>
       </c>
       <c r="K37" s="2">
         <f>J37-J37*Supuestos!$B$2-Supuestos!$B$3-F37</f>
@@ -3100,7 +3072,7 @@
       </c>
       <c r="I38" s="2" t="n"/>
       <c r="J38" s="3" t="n">
-        <v>107.99</v>
+        <v>109.99</v>
       </c>
       <c r="K38" s="2">
         <f>J38-J38*Supuestos!$B$2-Supuestos!$B$3-F38</f>
@@ -3167,7 +3139,7 @@
       </c>
       <c r="I39" s="2" t="n"/>
       <c r="J39" s="3" t="n">
-        <v>277.99</v>
+        <v>279.99</v>
       </c>
       <c r="K39" s="2">
         <f>J39-J39*Supuestos!$B$2-Supuestos!$B$3-F39</f>
@@ -3234,7 +3206,7 @@
       </c>
       <c r="I40" s="2" t="n"/>
       <c r="J40" s="3" t="n">
-        <v>58.99</v>
+        <v>61.99</v>
       </c>
       <c r="K40" s="2">
         <f>J40-J40*Supuestos!$B$2-Supuestos!$B$3-F40</f>
@@ -3301,7 +3273,7 @@
       </c>
       <c r="I41" s="2" t="n"/>
       <c r="J41" s="3" t="n">
-        <v>63.99</v>
+        <v>66.98999999999999</v>
       </c>
       <c r="K41" s="2">
         <f>J41-J41*Supuestos!$B$2-Supuestos!$B$3-F41</f>
@@ -3368,7 +3340,7 @@
       </c>
       <c r="I42" s="2" t="n"/>
       <c r="J42" s="3" t="n">
-        <v>61.99</v>
+        <v>63.99</v>
       </c>
       <c r="K42" s="2">
         <f>J42-J42*Supuestos!$B$2-Supuestos!$B$3-F42</f>
@@ -3435,7 +3407,7 @@
       </c>
       <c r="I43" s="2" t="n"/>
       <c r="J43" s="3" t="n">
-        <v>69.98999999999999</v>
+        <v>71.98999999999999</v>
       </c>
       <c r="K43" s="2">
         <f>J43-J43*Supuestos!$B$2-Supuestos!$B$3-F43</f>
@@ -3502,7 +3474,7 @@
       </c>
       <c r="I44" s="2" t="n"/>
       <c r="J44" s="3" t="n">
-        <v>60.99</v>
+        <v>62.99</v>
       </c>
       <c r="K44" s="2">
         <f>J44-J44*Supuestos!$B$2-Supuestos!$B$3-F44</f>
@@ -3569,7 +3541,7 @@
       </c>
       <c r="I45" s="2" t="n"/>
       <c r="J45" s="3" t="n">
-        <v>65.98999999999999</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="K45" s="2">
         <f>J45-J45*Supuestos!$B$2-Supuestos!$B$3-F45</f>
@@ -3636,7 +3608,7 @@
       </c>
       <c r="I46" s="2" t="n"/>
       <c r="J46" s="3" t="n">
-        <v>56.99</v>
+        <v>58.99</v>
       </c>
       <c r="K46" s="2">
         <f>J46-J46*Supuestos!$B$2-Supuestos!$B$3-F46</f>
@@ -3703,7 +3675,7 @@
       </c>
       <c r="I47" s="2" t="n"/>
       <c r="J47" s="3" t="n">
-        <v>58.99</v>
+        <v>61.99</v>
       </c>
       <c r="K47" s="2">
         <f>J47-J47*Supuestos!$B$2-Supuestos!$B$3-F47</f>
@@ -3770,7 +3742,7 @@
       </c>
       <c r="I48" s="2" t="n"/>
       <c r="J48" s="3" t="n">
-        <v>48.99</v>
+        <v>51.99</v>
       </c>
       <c r="K48" s="2">
         <f>J48-J48*Supuestos!$B$2-Supuestos!$B$3-F48</f>
@@ -3837,7 +3809,7 @@
       </c>
       <c r="I49" s="2" t="n"/>
       <c r="J49" s="3" t="n">
-        <v>28.99</v>
+        <v>30.99</v>
       </c>
       <c r="K49" s="2">
         <f>J49-J49*Supuestos!$B$2-Supuestos!$B$3-F49</f>
@@ -3904,7 +3876,7 @@
       </c>
       <c r="I50" s="2" t="n"/>
       <c r="J50" s="3" t="n">
-        <v>28.99</v>
+        <v>30.99</v>
       </c>
       <c r="K50" s="2">
         <f>J50-J50*Supuestos!$B$2-Supuestos!$B$3-F50</f>
@@ -3971,7 +3943,7 @@
       </c>
       <c r="I51" s="2" t="n"/>
       <c r="J51" s="3" t="n">
-        <v>38.99</v>
+        <v>40.99</v>
       </c>
       <c r="K51" s="2">
         <f>J51-J51*Supuestos!$B$2-Supuestos!$B$3-F51</f>
@@ -4035,7 +4007,7 @@
       </c>
       <c r="I52" s="2" t="n"/>
       <c r="J52" s="3" t="n">
-        <v>55.99</v>
+        <v>58.99</v>
       </c>
       <c r="K52" s="2">
         <f>J52-J52*Supuestos!$B$2-Supuestos!$B$3-F52</f>
@@ -4099,7 +4071,7 @@
       </c>
       <c r="I53" s="2" t="n"/>
       <c r="J53" s="3" t="n">
-        <v>38.99</v>
+        <v>40.99</v>
       </c>
       <c r="K53" s="2">
         <f>J53-J53*Supuestos!$B$2-Supuestos!$B$3-F53</f>
@@ -4163,7 +4135,7 @@
       </c>
       <c r="I54" s="2" t="n"/>
       <c r="J54" s="3" t="n">
-        <v>27.99</v>
+        <v>29.99</v>
       </c>
       <c r="K54" s="2">
         <f>J54-J54*Supuestos!$B$2-Supuestos!$B$3-F54</f>
@@ -4227,7 +4199,7 @@
       </c>
       <c r="I55" s="2" t="n"/>
       <c r="J55" s="3" t="n">
-        <v>31.99</v>
+        <v>33.99</v>
       </c>
       <c r="K55" s="2">
         <f>J55-J55*Supuestos!$B$2-Supuestos!$B$3-F55</f>
@@ -4291,7 +4263,7 @@
       </c>
       <c r="I56" s="2" t="n"/>
       <c r="J56" s="3" t="n">
-        <v>29.99</v>
+        <v>31.99</v>
       </c>
       <c r="K56" s="2">
         <f>J56-J56*Supuestos!$B$2-Supuestos!$B$3-F56</f>
@@ -4358,7 +4330,7 @@
       </c>
       <c r="I57" s="2" t="n"/>
       <c r="J57" s="3" t="n">
-        <v>29.99</v>
+        <v>31.99</v>
       </c>
       <c r="K57" s="2">
         <f>J57-J57*Supuestos!$B$2-Supuestos!$B$3-F57</f>
@@ -4425,7 +4397,7 @@
       </c>
       <c r="I58" s="2" t="n"/>
       <c r="J58" s="3" t="n">
-        <v>47.99</v>
+        <v>49.99</v>
       </c>
       <c r="K58" s="2">
         <f>J58-J58*Supuestos!$B$2-Supuestos!$B$3-F58</f>
@@ -4489,7 +4461,7 @@
       </c>
       <c r="I59" s="2" t="n"/>
       <c r="J59" s="3" t="n">
-        <v>41.99</v>
+        <v>43.99</v>
       </c>
       <c r="K59" s="2">
         <f>J59-J59*Supuestos!$B$2-Supuestos!$B$3-F59</f>
@@ -4553,7 +4525,7 @@
       </c>
       <c r="I60" s="2" t="n"/>
       <c r="J60" s="3" t="n">
-        <v>67.98999999999999</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="K60" s="2">
         <f>J60-J60*Supuestos!$B$2-Supuestos!$B$3-F60</f>
@@ -4617,7 +4589,7 @@
       </c>
       <c r="I61" s="2" t="n"/>
       <c r="J61" s="3" t="n">
-        <v>23.99</v>
+        <v>25.99</v>
       </c>
       <c r="K61" s="2">
         <f>J61-J61*Supuestos!$B$2-Supuestos!$B$3-F61</f>
@@ -4684,7 +4656,7 @@
       </c>
       <c r="I62" s="2" t="n"/>
       <c r="J62" s="3" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="K62" s="2">
         <f>J62-J62*Supuestos!$B$2-Supuestos!$B$3-F62</f>
@@ -4751,7 +4723,7 @@
       </c>
       <c r="I63" s="2" t="n"/>
       <c r="J63" s="3" t="n">
-        <v>33.99</v>
+        <v>35.99</v>
       </c>
       <c r="K63" s="2">
         <f>J63-J63*Supuestos!$B$2-Supuestos!$B$3-F63</f>
@@ -4828,7 +4800,7 @@
       <c r="L64" s="4" t="n"/>
       <c r="M64" s="2" t="n"/>
       <c r="N64" s="2" t="n"/>
-      <c r="O64" s="6" t="inlineStr">
+      <c r="O64" s="5" t="inlineStr">
         <is>
           <t>No vender suelto: el mercado está casi al precio de costo</t>
         </is>
@@ -4891,7 +4863,7 @@
       <c r="L65" s="4" t="n"/>
       <c r="M65" s="2" t="n"/>
       <c r="N65" s="2" t="n"/>
-      <c r="O65" s="6" t="inlineStr">
+      <c r="O65" s="5" t="inlineStr">
         <is>
           <t>No vender suelto: el mercado está casi al precio de costo</t>
         </is>
@@ -4954,7 +4926,7 @@
       <c r="L66" s="4" t="n"/>
       <c r="M66" s="2" t="n"/>
       <c r="N66" s="2" t="n"/>
-      <c r="O66" s="6" t="inlineStr">
+      <c r="O66" s="5" t="inlineStr">
         <is>
           <t>No vender suelto: el mercado está casi al precio de costo</t>
         </is>
@@ -5017,7 +4989,7 @@
       <c r="L67" s="4" t="n"/>
       <c r="M67" s="2" t="n"/>
       <c r="N67" s="2" t="n"/>
-      <c r="O67" s="6" t="inlineStr">
+      <c r="O67" s="5" t="inlineStr">
         <is>
           <t>No vender suelto: el mercado está casi al precio de costo</t>
         </is>
@@ -5080,7 +5052,7 @@
       <c r="L68" s="4" t="n"/>
       <c r="M68" s="2" t="n"/>
       <c r="N68" s="2" t="n"/>
-      <c r="O68" s="6" t="inlineStr">
+      <c r="O68" s="5" t="inlineStr">
         <is>
           <t>No vender suelto: el mercado está casi al precio de costo</t>
         </is>
@@ -5133,7 +5105,7 @@
       </c>
       <c r="I69" s="2" t="n"/>
       <c r="J69" s="3" t="n">
-        <v>72.98999999999999</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="K69" s="2">
         <f>J69-J69*Supuestos!$B$2-Supuestos!$B$3-F69</f>
@@ -5200,7 +5172,7 @@
       </c>
       <c r="I70" s="2" t="n"/>
       <c r="J70" s="3" t="n">
-        <v>72.98999999999999</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="K70" s="2">
         <f>J70-J70*Supuestos!$B$2-Supuestos!$B$3-F70</f>
@@ -5273,7 +5245,7 @@
         <v>23.49</v>
       </c>
       <c r="J71" s="3" t="n">
-        <v>23.99</v>
+        <v>25.99</v>
       </c>
       <c r="K71" s="2">
         <f>J71-J71*Supuestos!$B$2-Supuestos!$B$3-F71</f>
@@ -5344,7 +5316,7 @@
       </c>
       <c r="I72" s="2" t="n"/>
       <c r="J72" s="3" t="n">
-        <v>64.98999999999999</v>
+        <v>66.98999999999999</v>
       </c>
       <c r="K72" s="2">
         <f>J72-J72*Supuestos!$B$2-Supuestos!$B$3-F72</f>
@@ -5411,7 +5383,7 @@
       </c>
       <c r="I73" s="2" t="n"/>
       <c r="J73" s="3" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="K73" s="2">
         <f>J73-J73*Supuestos!$B$2-Supuestos!$B$3-F73</f>
@@ -5475,7 +5447,7 @@
       </c>
       <c r="I74" s="2" t="n"/>
       <c r="J74" s="3" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="K74" s="2">
         <f>J74-J74*Supuestos!$B$2-Supuestos!$B$3-F74</f>
@@ -5542,7 +5514,7 @@
       </c>
       <c r="I75" s="2" t="n"/>
       <c r="J75" s="3" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="K75" s="2">
         <f>J75-J75*Supuestos!$B$2-Supuestos!$B$3-F75</f>
@@ -5609,7 +5581,7 @@
       </c>
       <c r="I76" s="2" t="n"/>
       <c r="J76" s="3" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="K76" s="2">
         <f>J76-J76*Supuestos!$B$2-Supuestos!$B$3-F76</f>
@@ -5676,7 +5648,7 @@
       </c>
       <c r="I77" s="2" t="n"/>
       <c r="J77" s="3" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="K77" s="2">
         <f>J77-J77*Supuestos!$B$2-Supuestos!$B$3-F77</f>
@@ -5743,7 +5715,7 @@
       </c>
       <c r="I78" s="2" t="n"/>
       <c r="J78" s="3" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="K78" s="2">
         <f>J78-J78*Supuestos!$B$2-Supuestos!$B$3-F78</f>
@@ -5810,7 +5782,7 @@
       </c>
       <c r="I79" s="2" t="n"/>
       <c r="J79" s="3" t="n">
-        <v>34.99</v>
+        <v>36.99</v>
       </c>
       <c r="K79" s="2">
         <f>J79-J79*Supuestos!$B$2-Supuestos!$B$3-F79</f>
@@ -5877,7 +5849,7 @@
       </c>
       <c r="I80" s="2" t="n"/>
       <c r="J80" s="3" t="n">
-        <v>30.99</v>
+        <v>32.99</v>
       </c>
       <c r="K80" s="2">
         <f>J80-J80*Supuestos!$B$2-Supuestos!$B$3-F80</f>
@@ -5944,7 +5916,7 @@
       </c>
       <c r="I81" s="2" t="n"/>
       <c r="J81" s="3" t="n">
-        <v>27.99</v>
+        <v>29.99</v>
       </c>
       <c r="K81" s="2">
         <f>J81-J81*Supuestos!$B$2-Supuestos!$B$3-F81</f>
@@ -6011,7 +5983,7 @@
       </c>
       <c r="I82" s="2" t="n"/>
       <c r="J82" s="3" t="n">
-        <v>73.98999999999999</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="K82" s="2">
         <f>J82-J82*Supuestos!$B$2-Supuestos!$B$3-F82</f>
@@ -6078,7 +6050,7 @@
       </c>
       <c r="I83" s="2" t="n"/>
       <c r="J83" s="3" t="n">
-        <v>52.99</v>
+        <v>54.99</v>
       </c>
       <c r="K83" s="2">
         <f>J83-J83*Supuestos!$B$2-Supuestos!$B$3-F83</f>
@@ -6145,7 +6117,7 @@
       </c>
       <c r="I84" s="2" t="n"/>
       <c r="J84" s="3" t="n">
-        <v>66.98999999999999</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="K84" s="2">
         <f>J84-J84*Supuestos!$B$2-Supuestos!$B$3-F84</f>
@@ -6212,7 +6184,7 @@
       </c>
       <c r="I85" s="2" t="n"/>
       <c r="J85" s="3" t="n">
-        <v>56.99</v>
+        <v>58.99</v>
       </c>
       <c r="K85" s="2">
         <f>J85-J85*Supuestos!$B$2-Supuestos!$B$3-F85</f>
@@ -6279,7 +6251,7 @@
       </c>
       <c r="I86" s="2" t="n"/>
       <c r="J86" s="3" t="n">
-        <v>37.99</v>
+        <v>39.99</v>
       </c>
       <c r="K86" s="2">
         <f>J86-J86*Supuestos!$B$2-Supuestos!$B$3-F86</f>
@@ -6346,7 +6318,7 @@
       </c>
       <c r="I87" s="2" t="n"/>
       <c r="J87" s="3" t="n">
-        <v>56.99</v>
+        <v>59.99</v>
       </c>
       <c r="K87" s="2">
         <f>J87-J87*Supuestos!$B$2-Supuestos!$B$3-F87</f>
@@ -6417,7 +6389,7 @@
       </c>
       <c r="I88" s="2" t="n"/>
       <c r="J88" s="3" t="n">
-        <v>56.99</v>
+        <v>59.99</v>
       </c>
       <c r="K88" s="2">
         <f>J88-J88*Supuestos!$B$2-Supuestos!$B$3-F88</f>
@@ -6488,7 +6460,7 @@
       </c>
       <c r="I89" s="2" t="n"/>
       <c r="J89" s="3" t="n">
-        <v>120.99</v>
+        <v>122.99</v>
       </c>
       <c r="K89" s="2">
         <f>J89-J89*Supuestos!$B$2-Supuestos!$B$3-F89</f>
@@ -6555,7 +6527,7 @@
       </c>
       <c r="I90" s="2" t="n"/>
       <c r="J90" s="3" t="n">
-        <v>33.99</v>
+        <v>35.99</v>
       </c>
       <c r="K90" s="2">
         <f>J90-J90*Supuestos!$B$2-Supuestos!$B$3-F90</f>
@@ -6622,7 +6594,7 @@
       </c>
       <c r="I91" s="2" t="n"/>
       <c r="J91" s="3" t="n">
-        <v>88.98999999999999</v>
+        <v>91.98999999999999</v>
       </c>
       <c r="K91" s="2">
         <f>J91-J91*Supuestos!$B$2-Supuestos!$B$3-F91</f>
@@ -6689,7 +6661,7 @@
       </c>
       <c r="I92" s="2" t="n"/>
       <c r="J92" s="3" t="n">
-        <v>50.99</v>
+        <v>53.99</v>
       </c>
       <c r="K92" s="2">
         <f>J92-J92*Supuestos!$B$2-Supuestos!$B$3-F92</f>
@@ -6756,7 +6728,7 @@
       </c>
       <c r="I93" s="2" t="n"/>
       <c r="J93" s="3" t="n">
-        <v>145.99</v>
+        <v>148.99</v>
       </c>
       <c r="K93" s="2">
         <f>J93-J93*Supuestos!$B$2-Supuestos!$B$3-F93</f>
@@ -6823,7 +6795,7 @@
       </c>
       <c r="I94" s="2" t="n"/>
       <c r="J94" s="3" t="n">
-        <v>360.99</v>
+        <v>362.99</v>
       </c>
       <c r="K94" s="2">
         <f>J94-J94*Supuestos!$B$2-Supuestos!$B$3-F94</f>
@@ -6890,7 +6862,7 @@
       </c>
       <c r="I95" s="2" t="n"/>
       <c r="J95" s="3" t="n">
-        <v>147.99</v>
+        <v>149.99</v>
       </c>
       <c r="K95" s="2">
         <f>J95-J95*Supuestos!$B$2-Supuestos!$B$3-F95</f>
@@ -6957,7 +6929,7 @@
       </c>
       <c r="I96" s="2" t="n"/>
       <c r="J96" s="3" t="n">
-        <v>147.99</v>
+        <v>149.99</v>
       </c>
       <c r="K96" s="2">
         <f>J96-J96*Supuestos!$B$2-Supuestos!$B$3-F96</f>
@@ -7024,7 +6996,7 @@
       </c>
       <c r="I97" s="2" t="n"/>
       <c r="J97" s="3" t="n">
-        <v>495.99</v>
+        <v>498.99</v>
       </c>
       <c r="K97" s="2">
         <f>J97-J97*Supuestos!$B$2-Supuestos!$B$3-F97</f>
@@ -7091,7 +7063,7 @@
       </c>
       <c r="I98" s="2" t="n"/>
       <c r="J98" s="3" t="n">
-        <v>259.99</v>
+        <v>262.99</v>
       </c>
       <c r="K98" s="2">
         <f>J98-J98*Supuestos!$B$2-Supuestos!$B$3-F98</f>
@@ -7158,7 +7130,7 @@
       </c>
       <c r="I99" s="2" t="n"/>
       <c r="J99" s="3" t="n">
-        <v>105.99</v>
+        <v>107.99</v>
       </c>
       <c r="K99" s="2">
         <f>J99-J99*Supuestos!$B$2-Supuestos!$B$3-F99</f>
@@ -7225,7 +7197,7 @@
       </c>
       <c r="I100" s="2" t="n"/>
       <c r="J100" s="3" t="n">
-        <v>280.99</v>
+        <v>282.99</v>
       </c>
       <c r="K100" s="2">
         <f>J100-J100*Supuestos!$B$2-Supuestos!$B$3-F100</f>
@@ -7292,7 +7264,7 @@
       </c>
       <c r="I101" s="2" t="n"/>
       <c r="J101" s="3" t="n">
-        <v>94.98999999999999</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="K101" s="2">
         <f>J101-J101*Supuestos!$B$2-Supuestos!$B$3-F101</f>
@@ -7359,7 +7331,7 @@
       </c>
       <c r="I102" s="2" t="n"/>
       <c r="J102" s="3" t="n">
-        <v>304.99</v>
+        <v>306.99</v>
       </c>
       <c r="K102" s="2">
         <f>J102-J102*Supuestos!$B$2-Supuestos!$B$3-F102</f>
@@ -7426,7 +7398,7 @@
       </c>
       <c r="I103" s="2" t="n"/>
       <c r="J103" s="3" t="n">
-        <v>26.99</v>
+        <v>28.99</v>
       </c>
       <c r="K103" s="2">
         <f>J103-J103*Supuestos!$B$2-Supuestos!$B$3-F103</f>
@@ -7493,7 +7465,7 @@
       </c>
       <c r="I104" s="2" t="n"/>
       <c r="J104" s="3" t="n">
-        <v>56.99</v>
+        <v>58.99</v>
       </c>
       <c r="K104" s="2">
         <f>J104-J104*Supuestos!$B$2-Supuestos!$B$3-F104</f>
@@ -7560,7 +7532,7 @@
       </c>
       <c r="I105" s="2" t="n"/>
       <c r="J105" s="3" t="n">
-        <v>60.99</v>
+        <v>62.99</v>
       </c>
       <c r="K105" s="2">
         <f>J105-J105*Supuestos!$B$2-Supuestos!$B$3-F105</f>
@@ -7627,7 +7599,7 @@
       </c>
       <c r="I106" s="2" t="n"/>
       <c r="J106" s="3" t="n">
-        <v>44.99</v>
+        <v>46.99</v>
       </c>
       <c r="K106" s="2">
         <f>J106-J106*Supuestos!$B$2-Supuestos!$B$3-F106</f>
@@ -7691,7 +7663,7 @@
       </c>
       <c r="I107" s="2" t="n"/>
       <c r="J107" s="3" t="n">
-        <v>109.99</v>
+        <v>111.99</v>
       </c>
       <c r="K107" s="2">
         <f>J107-J107*Supuestos!$B$2-Supuestos!$B$3-F107</f>
@@ -7758,7 +7730,7 @@
       </c>
       <c r="I108" s="2" t="n"/>
       <c r="J108" s="3" t="n">
-        <v>109.99</v>
+        <v>111.99</v>
       </c>
       <c r="K108" s="2">
         <f>J108-J108*Supuestos!$B$2-Supuestos!$B$3-F108</f>
@@ -7825,7 +7797,7 @@
       </c>
       <c r="I109" s="2" t="n"/>
       <c r="J109" s="3" t="n">
-        <v>109.99</v>
+        <v>111.99</v>
       </c>
       <c r="K109" s="2">
         <f>J109-J109*Supuestos!$B$2-Supuestos!$B$3-F109</f>
@@ -7892,7 +7864,7 @@
       </c>
       <c r="I110" s="2" t="n"/>
       <c r="J110" s="3" t="n">
-        <v>109.99</v>
+        <v>111.99</v>
       </c>
       <c r="K110" s="2">
         <f>J110-J110*Supuestos!$B$2-Supuestos!$B$3-F110</f>
@@ -7959,7 +7931,7 @@
       </c>
       <c r="I111" s="2" t="n"/>
       <c r="J111" s="3" t="n">
-        <v>25.99</v>
+        <v>27.99</v>
       </c>
       <c r="K111" s="2">
         <f>J111-J111*Supuestos!$B$2-Supuestos!$B$3-F111</f>
@@ -8026,7 +7998,7 @@
       </c>
       <c r="I112" s="2" t="n"/>
       <c r="J112" s="3" t="n">
-        <v>28.99</v>
+        <v>30.99</v>
       </c>
       <c r="K112" s="2">
         <f>J112-J112*Supuestos!$B$2-Supuestos!$B$3-F112</f>
@@ -8093,7 +8065,7 @@
       </c>
       <c r="I113" s="2" t="n"/>
       <c r="J113" s="3" t="n">
-        <v>27.99</v>
+        <v>29.99</v>
       </c>
       <c r="K113" s="2">
         <f>J113-J113*Supuestos!$B$2-Supuestos!$B$3-F113</f>
@@ -8160,7 +8132,7 @@
       </c>
       <c r="I114" s="2" t="n"/>
       <c r="J114" s="3" t="n">
-        <v>55.99</v>
+        <v>57.99</v>
       </c>
       <c r="K114" s="2">
         <f>J114-J114*Supuestos!$B$2-Supuestos!$B$3-F114</f>
@@ -8227,7 +8199,7 @@
       </c>
       <c r="I115" s="2" t="n"/>
       <c r="J115" s="3" t="n">
-        <v>55.99</v>
+        <v>57.99</v>
       </c>
       <c r="K115" s="2">
         <f>J115-J115*Supuestos!$B$2-Supuestos!$B$3-F115</f>
@@ -8294,7 +8266,7 @@
       </c>
       <c r="I116" s="2" t="n"/>
       <c r="J116" s="3" t="n">
-        <v>56.99</v>
+        <v>58.99</v>
       </c>
       <c r="K116" s="2">
         <f>J116-J116*Supuestos!$B$2-Supuestos!$B$3-F116</f>
@@ -8416,11 +8388,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.6</v>
+        <v>7.5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Etiqueta + empaque. Si el precio incluye envío gratis, se suma al costo.</t>
+          <t>Etiqueta promedio nacional (USPS Ground Advantage, menos de 1 lb: unos $5.50 a $8.40 según la zona) + empaque. Si el precio incluye envío gratis, se suma al costo.</t>
         </is>
       </c>
     </row>
@@ -8431,7 +8403,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6.5</v>
+        <v>9.5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Precios EE. UU.: competencia puesta en la puerta (precio + envío promedio), ganancia mínima 10 USD, mensaje de entrega a la puerta
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp6cWLHDTqXsEaejCBC2fh
</commit_message>
<xml_diff>
--- a/us-filter-store/precios/precios-de-venta.xlsx
+++ b/us-filter-store/precios/precios-de-venta.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T116"/>
+  <dimension ref="A1:U116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -469,7 +469,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="9" customWidth="1" min="12" max="12"/>
@@ -481,6 +481,7 @@
     <col width="8" customWidth="1" min="18" max="18"/>
     <col width="40" customWidth="1" min="19" max="19"/>
     <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
@@ -526,7 +527,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Precio de la calle (mercado)</t>
+          <t>Calle puesta en la puerta (precio visto + envío promedio)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -581,7 +582,12 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Costo máximo del proveedor para ganar el mínimo vendiendo al precio de la calle</t>
+          <t>Costo máximo del proveedor para ganar el mínimo vendiendo al precio de la calle puesto en la puerta</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Precio de la calle sin envío (visto)</t>
         </is>
       </c>
     </row>
@@ -638,6 +644,7 @@
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -674,8 +681,9 @@
         <f>ROUNDUP(MAX((F3+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F3+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I3" s="2" t="n">
-        <v>44</v>
+      <c r="I3" s="2">
+        <f>U3+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J3" s="3" t="n">
         <v>46.99</v>
@@ -696,9 +704,9 @@
         <f>M3-M3*Supuestos!$B$2-Supuestos!$B$3-2*E3-Supuestos!$B$6</f>
         <v/>
       </c>
-      <c r="O3" s="5" t="inlineStr">
-        <is>
-          <t>Un poco sobre el mercado: aceptable con envío gratis y buen servicio</t>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Competitivo</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -719,6 +727,9 @@
         <f>(I3*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
       </c>
+      <c r="U3" s="2" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -755,17 +766,32 @@
         <f>ROUNDUP(MAX((F4+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F4+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I4" s="2" t="n">
-        <v>34.99</v>
-      </c>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="n"/>
-      <c r="O4" s="6" t="inlineStr">
-        <is>
-          <t>No competitivo: solo lo vendes ganando el mínimo si bajas el costo (ver última columna)</t>
+      <c r="I4" s="2">
+        <f>U4+Supuestos!$B$10</f>
+        <v/>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="K4" s="2">
+        <f>J4-J4*Supuestos!$B$2-Supuestos!$B$3-F4</f>
+        <v/>
+      </c>
+      <c r="L4" s="4">
+        <f>K4/J4</f>
+        <v/>
+      </c>
+      <c r="M4" s="2">
+        <f>ROUNDUP(MAX(2*J4*0.92,(2*E4+Supuestos!$B$6+Supuestos!$B$3+8)/(1-Supuestos!$B$2)),0)-0.01</f>
+        <v/>
+      </c>
+      <c r="N4" s="2">
+        <f>M4-M4*Supuestos!$B$2-Supuestos!$B$3-2*E4-Supuestos!$B$6</f>
+        <v/>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>Un poco sobre el mercado: lo compensa la entrega hasta la puerta</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -786,6 +812,9 @@
         <f>(I4*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
       </c>
+      <c r="U4" s="2" t="n">
+        <v>34.99</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -822,17 +851,32 @@
         <f>ROUNDUP(MAX((F5+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F5+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I5" s="2" t="n">
-        <v>36.99</v>
-      </c>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="2" t="n"/>
-      <c r="L5" s="4" t="n"/>
-      <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="n"/>
-      <c r="O5" s="6" t="inlineStr">
-        <is>
-          <t>No competitivo: solo lo vendes ganando el mínimo si bajas el costo (ver última columna)</t>
+      <c r="I5" s="2">
+        <f>U5+Supuestos!$B$10</f>
+        <v/>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="K5" s="2">
+        <f>J5-J5*Supuestos!$B$2-Supuestos!$B$3-F5</f>
+        <v/>
+      </c>
+      <c r="L5" s="4">
+        <f>K5/J5</f>
+        <v/>
+      </c>
+      <c r="M5" s="2">
+        <f>ROUNDUP(MAX(2*J5*0.92,(2*E5+Supuestos!$B$6+Supuestos!$B$3+8)/(1-Supuestos!$B$2)),0)-0.01</f>
+        <v/>
+      </c>
+      <c r="N5" s="2">
+        <f>M5-M5*Supuestos!$B$2-Supuestos!$B$3-2*E5-Supuestos!$B$6</f>
+        <v/>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>Un poco sobre el mercado: lo compensa la entrega hasta la puerta</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -853,6 +897,9 @@
         <f>(I5*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
       </c>
+      <c r="U5" s="2" t="n">
+        <v>36.99</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -889,8 +936,9 @@
         <f>ROUNDUP(MAX((F6+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F6+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I6" s="2" t="n">
-        <v>19</v>
+      <c r="I6" s="2">
+        <f>U6+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J6" s="3" t="n"/>
       <c r="K6" s="2" t="n"/>
@@ -899,7 +947,7 @@
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="6" t="inlineStr">
         <is>
-          <t>No competitivo: solo lo vendes ganando el mínimo si bajas el costo (ver última columna)</t>
+          <t>No competitivo: baja el costo con el proveedor (ver columna «Costo máximo»)</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -920,6 +968,9 @@
         <f>(I6*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
       </c>
+      <c r="U6" s="2" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -956,8 +1007,9 @@
         <f>ROUNDUP(MAX((F7+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F7+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I7" s="2" t="n">
-        <v>54.99</v>
+      <c r="I7" s="2">
+        <f>U7+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J7" s="3" t="n">
         <v>61.99</v>
@@ -978,9 +1030,9 @@
         <f>M7-M7*Supuestos!$B$2-Supuestos!$B$3-2*E7-Supuestos!$B$6</f>
         <v/>
       </c>
-      <c r="O7" s="5" t="inlineStr">
-        <is>
-          <t>Un poco sobre el mercado: aceptable con envío gratis y buen servicio</t>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Competitivo</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1001,6 +1053,9 @@
         <f>(I7*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
       </c>
+      <c r="U7" s="2" t="n">
+        <v>54.99</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1037,8 +1092,9 @@
         <f>ROUNDUP(MAX((F8+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F8+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I8" s="2" t="n">
-        <v>54.97</v>
+      <c r="I8" s="2">
+        <f>U8+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J8" s="3" t="n">
         <v>60.99</v>
@@ -1059,9 +1115,9 @@
         <f>M8-M8*Supuestos!$B$2-Supuestos!$B$3-2*E8-Supuestos!$B$6</f>
         <v/>
       </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>Un poco sobre el mercado: aceptable con envío gratis y buen servicio</t>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Competitivo</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1082,6 +1138,9 @@
         <f>(I8*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
       </c>
+      <c r="U8" s="2" t="n">
+        <v>54.97</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1118,17 +1177,32 @@
         <f>ROUNDUP(MAX((F9+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F9+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I9" s="2" t="n">
-        <v>49.99</v>
-      </c>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="4" t="n"/>
-      <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="n"/>
-      <c r="O9" s="6" t="inlineStr">
-        <is>
-          <t>No competitivo: solo lo vendes ganando el mínimo si bajas el costo (ver última columna)</t>
+      <c r="I9" s="2">
+        <f>U9+Supuestos!$B$10</f>
+        <v/>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>60.99</v>
+      </c>
+      <c r="K9" s="2">
+        <f>J9-J9*Supuestos!$B$2-Supuestos!$B$3-F9</f>
+        <v/>
+      </c>
+      <c r="L9" s="4">
+        <f>K9/J9</f>
+        <v/>
+      </c>
+      <c r="M9" s="2">
+        <f>ROUNDUP(MAX(2*J9*0.92,(2*E9+Supuestos!$B$6+Supuestos!$B$3+8)/(1-Supuestos!$B$2)),0)-0.01</f>
+        <v/>
+      </c>
+      <c r="N9" s="2">
+        <f>M9-M9*Supuestos!$B$2-Supuestos!$B$3-2*E9-Supuestos!$B$6</f>
+        <v/>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>Un poco sobre el mercado: lo compensa la entrega hasta la puerta</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1148,6 +1222,9 @@
       <c r="T9" s="2">
         <f>(I9*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>49.99</v>
       </c>
     </row>
     <row r="10">
@@ -1211,6 +1288,7 @@
         </is>
       </c>
       <c r="T10" s="2" t="n"/>
+      <c r="U10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1247,8 +1325,9 @@
         <f>ROUNDUP(MAX((F11+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F11+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I11" s="2" t="n">
-        <v>54.99</v>
+      <c r="I11" s="2">
+        <f>U11+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J11" s="3" t="n">
         <v>60.99</v>
@@ -1269,9 +1348,9 @@
         <f>M11-M11*Supuestos!$B$2-Supuestos!$B$3-2*E11-Supuestos!$B$6</f>
         <v/>
       </c>
-      <c r="O11" s="5" t="inlineStr">
-        <is>
-          <t>Un poco sobre el mercado: aceptable con envío gratis y buen servicio</t>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Competitivo</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1292,6 +1371,9 @@
         <f>(I11*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
       </c>
+      <c r="U11" s="2" t="n">
+        <v>54.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1328,8 +1410,9 @@
         <f>ROUNDUP(MAX((F12+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F12+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I12" s="2" t="n">
-        <v>54.99</v>
+      <c r="I12" s="2">
+        <f>U12+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J12" s="3" t="n">
         <v>57.99</v>
@@ -1350,9 +1433,9 @@
         <f>M12-M12*Supuestos!$B$2-Supuestos!$B$3-2*E12-Supuestos!$B$6</f>
         <v/>
       </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>Un poco sobre el mercado: aceptable con envío gratis y buen servicio</t>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Competitivo</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1372,6 +1455,9 @@
       <c r="T12" s="2">
         <f>(I12*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>54.99</v>
       </c>
     </row>
     <row r="13">
@@ -1435,6 +1521,7 @@
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" s="2" t="n"/>
+      <c r="U13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1489,6 +1576,7 @@
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" s="2" t="n"/>
+      <c r="U14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1525,8 +1613,9 @@
         <f>ROUNDUP(MAX((F15+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F15+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I15" s="2" t="n">
-        <v>45</v>
+      <c r="I15" s="2">
+        <f>U15+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="2" t="n"/>
@@ -1535,7 +1624,7 @@
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>No competitivo: solo lo vendes ganando el mínimo si bajas el costo (ver última columna)</t>
+          <t>No competitivo: baja el costo con el proveedor (ver columna «Costo máximo»)</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1555,6 +1644,9 @@
       <c r="T15" s="2">
         <f>(I15*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
+      </c>
+      <c r="U15" s="2" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="16">
@@ -1618,6 +1710,7 @@
         </is>
       </c>
       <c r="T16" s="2" t="n"/>
+      <c r="U16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1672,6 +1765,7 @@
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" s="2" t="n"/>
+      <c r="U17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1726,6 +1820,7 @@
       </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" s="2" t="n"/>
+      <c r="U18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1780,6 +1875,7 @@
       </c>
       <c r="S19" t="inlineStr"/>
       <c r="T19" s="2" t="n"/>
+      <c r="U19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1834,6 +1930,7 @@
       </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" s="2" t="n"/>
+      <c r="U20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1888,6 +1985,7 @@
       </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" s="2" t="n"/>
+      <c r="U21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1942,6 +2040,7 @@
       </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" s="2" t="n"/>
+      <c r="U22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1996,6 +2095,7 @@
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" s="2" t="n"/>
+      <c r="U23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2050,6 +2150,7 @@
       </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" s="2" t="n"/>
+      <c r="U24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2104,6 +2205,7 @@
       </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" s="2" t="n"/>
+      <c r="U25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2158,6 +2260,7 @@
       </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" s="2" t="n"/>
+      <c r="U26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2212,6 +2315,7 @@
       </c>
       <c r="S27" t="inlineStr"/>
       <c r="T27" s="2" t="n"/>
+      <c r="U27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2266,6 +2370,7 @@
       </c>
       <c r="S28" t="inlineStr"/>
       <c r="T28" s="2" t="n"/>
+      <c r="U28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2320,6 +2425,7 @@
       </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" s="2" t="n"/>
+      <c r="U29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2374,6 +2480,7 @@
       </c>
       <c r="S30" t="inlineStr"/>
       <c r="T30" s="2" t="n"/>
+      <c r="U30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2428,6 +2535,7 @@
       </c>
       <c r="S31" t="inlineStr"/>
       <c r="T31" s="2" t="n"/>
+      <c r="U31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2482,6 +2590,7 @@
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" s="2" t="n"/>
+      <c r="U32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2536,6 +2645,7 @@
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" s="2" t="n"/>
+      <c r="U33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2590,6 +2700,7 @@
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" s="2" t="n"/>
+      <c r="U34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2644,6 +2755,7 @@
       </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" s="2" t="n"/>
+      <c r="U35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2698,6 +2810,7 @@
       </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" s="2" t="n"/>
+      <c r="U36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2752,6 +2865,7 @@
       </c>
       <c r="S37" t="inlineStr"/>
       <c r="T37" s="2" t="n"/>
+      <c r="U37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2806,6 +2920,7 @@
       </c>
       <c r="S38" t="inlineStr"/>
       <c r="T38" s="2" t="n"/>
+      <c r="U38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2860,6 +2975,7 @@
       </c>
       <c r="S39" t="inlineStr"/>
       <c r="T39" s="2" t="n"/>
+      <c r="U39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2914,6 +3030,7 @@
       </c>
       <c r="S40" t="inlineStr"/>
       <c r="T40" s="2" t="n"/>
+      <c r="U40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2968,6 +3085,7 @@
       </c>
       <c r="S41" t="inlineStr"/>
       <c r="T41" s="2" t="n"/>
+      <c r="U41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3022,6 +3140,7 @@
       </c>
       <c r="S42" t="inlineStr"/>
       <c r="T42" s="2" t="n"/>
+      <c r="U42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3076,6 +3195,7 @@
       </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" s="2" t="n"/>
+      <c r="U43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3130,6 +3250,7 @@
       </c>
       <c r="S44" t="inlineStr"/>
       <c r="T44" s="2" t="n"/>
+      <c r="U44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3184,6 +3305,7 @@
       </c>
       <c r="S45" t="inlineStr"/>
       <c r="T45" s="2" t="n"/>
+      <c r="U45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3238,6 +3360,7 @@
       </c>
       <c r="S46" t="inlineStr"/>
       <c r="T46" s="2" t="n"/>
+      <c r="U46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3292,6 +3415,7 @@
       </c>
       <c r="S47" t="inlineStr"/>
       <c r="T47" s="2" t="n"/>
+      <c r="U47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3346,6 +3470,7 @@
       </c>
       <c r="S48" t="inlineStr"/>
       <c r="T48" s="2" t="n"/>
+      <c r="U48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3400,6 +3525,7 @@
       </c>
       <c r="S49" t="inlineStr"/>
       <c r="T49" s="2" t="n"/>
+      <c r="U49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3454,6 +3580,7 @@
       </c>
       <c r="S50" t="inlineStr"/>
       <c r="T50" s="2" t="n"/>
+      <c r="U50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3505,6 +3632,7 @@
       <c r="Q51" t="inlineStr"/>
       <c r="S51" t="inlineStr"/>
       <c r="T51" s="2" t="n"/>
+      <c r="U51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3556,6 +3684,7 @@
       <c r="Q52" t="inlineStr"/>
       <c r="S52" t="inlineStr"/>
       <c r="T52" s="2" t="n"/>
+      <c r="U52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3607,6 +3736,7 @@
       <c r="Q53" t="inlineStr"/>
       <c r="S53" t="inlineStr"/>
       <c r="T53" s="2" t="n"/>
+      <c r="U53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3658,6 +3788,7 @@
       <c r="Q54" t="inlineStr"/>
       <c r="S54" t="inlineStr"/>
       <c r="T54" s="2" t="n"/>
+      <c r="U54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3709,6 +3840,7 @@
       <c r="Q55" t="inlineStr"/>
       <c r="S55" t="inlineStr"/>
       <c r="T55" s="2" t="n"/>
+      <c r="U55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3763,6 +3895,7 @@
       </c>
       <c r="S56" t="inlineStr"/>
       <c r="T56" s="2" t="n"/>
+      <c r="U56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3817,6 +3950,7 @@
       </c>
       <c r="S57" t="inlineStr"/>
       <c r="T57" s="2" t="n"/>
+      <c r="U57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3868,6 +4002,7 @@
       <c r="Q58" t="inlineStr"/>
       <c r="S58" t="inlineStr"/>
       <c r="T58" s="2" t="n"/>
+      <c r="U58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3919,6 +4054,7 @@
       <c r="Q59" t="inlineStr"/>
       <c r="S59" t="inlineStr"/>
       <c r="T59" s="2" t="n"/>
+      <c r="U59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3970,6 +4106,7 @@
       <c r="Q60" t="inlineStr"/>
       <c r="S60" t="inlineStr"/>
       <c r="T60" s="2" t="n"/>
+      <c r="U60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4024,6 +4161,7 @@
       </c>
       <c r="S61" t="inlineStr"/>
       <c r="T61" s="2" t="n"/>
+      <c r="U61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4078,6 +4216,7 @@
       </c>
       <c r="S62" t="inlineStr"/>
       <c r="T62" s="2" t="n"/>
+      <c r="U62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4132,6 +4271,7 @@
       </c>
       <c r="S63" t="inlineStr"/>
       <c r="T63" s="2" t="n"/>
+      <c r="U63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4168,8 +4308,9 @@
         <f>ROUNDUP(MAX((F64+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F64+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I64" s="2" t="n">
-        <v>49.98</v>
+      <c r="I64" s="2">
+        <f>U64+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J64" s="3" t="n"/>
       <c r="K64" s="2" t="n"/>
@@ -4178,7 +4319,7 @@
       <c r="N64" s="2" t="n"/>
       <c r="O64" s="6" t="inlineStr">
         <is>
-          <t>No competitivo: solo lo vendes ganando el mínimo si bajas el costo (ver última columna)</t>
+          <t>No competitivo: baja el costo con el proveedor (ver columna «Costo máximo»)</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
@@ -4199,6 +4340,9 @@
         <f>(I64*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
       </c>
+      <c r="U64" s="2" t="n">
+        <v>49.98</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4235,8 +4379,9 @@
         <f>ROUNDUP(MAX((F65+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F65+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I65" s="2" t="n">
-        <v>49.49</v>
+      <c r="I65" s="2">
+        <f>U65+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J65" s="3" t="n"/>
       <c r="K65" s="2" t="n"/>
@@ -4245,7 +4390,7 @@
       <c r="N65" s="2" t="n"/>
       <c r="O65" s="6" t="inlineStr">
         <is>
-          <t>No competitivo: solo lo vendes ganando el mínimo si bajas el costo (ver última columna)</t>
+          <t>No competitivo: baja el costo con el proveedor (ver columna «Costo máximo»)</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -4266,6 +4411,9 @@
         <f>(I65*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
       </c>
+      <c r="U65" s="2" t="n">
+        <v>49.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4302,8 +4450,9 @@
         <f>ROUNDUP(MAX((F66+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F66+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I66" s="2" t="n">
-        <v>49.49</v>
+      <c r="I66" s="2">
+        <f>U66+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J66" s="3" t="n"/>
       <c r="K66" s="2" t="n"/>
@@ -4312,7 +4461,7 @@
       <c r="N66" s="2" t="n"/>
       <c r="O66" s="6" t="inlineStr">
         <is>
-          <t>No competitivo: solo lo vendes ganando el mínimo si bajas el costo (ver última columna)</t>
+          <t>No competitivo: baja el costo con el proveedor (ver columna «Costo máximo»)</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -4333,6 +4482,9 @@
         <f>(I66*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
       </c>
+      <c r="U66" s="2" t="n">
+        <v>49.49</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4369,8 +4521,9 @@
         <f>ROUNDUP(MAX((F67+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F67+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I67" s="2" t="n">
-        <v>49.49</v>
+      <c r="I67" s="2">
+        <f>U67+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J67" s="3" t="n"/>
       <c r="K67" s="2" t="n"/>
@@ -4379,7 +4532,7 @@
       <c r="N67" s="2" t="n"/>
       <c r="O67" s="6" t="inlineStr">
         <is>
-          <t>No competitivo: solo lo vendes ganando el mínimo si bajas el costo (ver última columna)</t>
+          <t>No competitivo: baja el costo con el proveedor (ver columna «Costo máximo»)</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -4400,6 +4553,9 @@
         <f>(I67*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
       </c>
+      <c r="U67" s="2" t="n">
+        <v>49.49</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4436,8 +4592,9 @@
         <f>ROUNDUP(MAX((F68+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F68+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I68" s="2" t="n">
-        <v>49.95</v>
+      <c r="I68" s="2">
+        <f>U68+Supuestos!$B$10</f>
+        <v/>
       </c>
       <c r="J68" s="3" t="n"/>
       <c r="K68" s="2" t="n"/>
@@ -4446,7 +4603,7 @@
       <c r="N68" s="2" t="n"/>
       <c r="O68" s="6" t="inlineStr">
         <is>
-          <t>No competitivo: solo lo vendes ganando el mínimo si bajas el costo (ver última columna)</t>
+          <t>No competitivo: baja el costo con el proveedor (ver columna «Costo máximo»)</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -4466,6 +4623,9 @@
       <c r="T68" s="2">
         <f>(I68*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
+      </c>
+      <c r="U68" s="2" t="n">
+        <v>49.95</v>
       </c>
     </row>
     <row r="69">
@@ -4521,6 +4681,7 @@
       </c>
       <c r="S69" t="inlineStr"/>
       <c r="T69" s="2" t="n"/>
+      <c r="U69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4575,6 +4736,7 @@
       </c>
       <c r="S70" t="inlineStr"/>
       <c r="T70" s="2" t="n"/>
+      <c r="U70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4611,17 +4773,32 @@
         <f>ROUNDUP(MAX((F71+Supuestos!$B$3)/(1-Supuestos!$B$2-Supuestos!$B$8),(F71+Supuestos!$B$3+Supuestos!$B$7)/(1-Supuestos!$B$2)),0)-0.01</f>
         <v/>
       </c>
-      <c r="I71" s="2" t="n">
-        <v>23.49</v>
-      </c>
-      <c r="J71" s="3" t="n"/>
-      <c r="K71" s="2" t="n"/>
-      <c r="L71" s="4" t="n"/>
-      <c r="M71" s="2" t="n"/>
-      <c r="N71" s="2" t="n"/>
-      <c r="O71" s="6" t="inlineStr">
-        <is>
-          <t>No competitivo: solo lo vendes ganando el mínimo si bajas el costo (ver última columna)</t>
+      <c r="I71" s="2">
+        <f>U71+Supuestos!$B$10</f>
+        <v/>
+      </c>
+      <c r="J71" s="3" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="K71" s="2">
+        <f>J71-J71*Supuestos!$B$2-Supuestos!$B$3-F71</f>
+        <v/>
+      </c>
+      <c r="L71" s="4">
+        <f>K71/J71</f>
+        <v/>
+      </c>
+      <c r="M71" s="2">
+        <f>ROUNDUP(MAX(2*J71*0.92,(2*E71+Supuestos!$B$6+Supuestos!$B$3+8)/(1-Supuestos!$B$2)),0)-0.01</f>
+        <v/>
+      </c>
+      <c r="N71" s="2">
+        <f>M71-M71*Supuestos!$B$2-Supuestos!$B$3-2*E71-Supuestos!$B$6</f>
+        <v/>
+      </c>
+      <c r="O71" s="5" t="inlineStr">
+        <is>
+          <t>Un poco sobre el mercado: lo compensa la entrega hasta la puerta</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -4641,6 +4818,9 @@
       <c r="T71" s="2">
         <f>(I71*(1-Supuestos!$B$2)-Supuestos!$B$3-Supuestos!$B$5-Supuestos!$B$9)/(1+Supuestos!$B$4)</f>
         <v/>
+      </c>
+      <c r="U71" s="2" t="n">
+        <v>23.49</v>
       </c>
     </row>
     <row r="72">
@@ -4696,6 +4876,7 @@
       </c>
       <c r="S72" t="inlineStr"/>
       <c r="T72" s="2" t="n"/>
+      <c r="U72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4747,6 +4928,7 @@
       <c r="Q73" t="inlineStr"/>
       <c r="S73" t="inlineStr"/>
       <c r="T73" s="2" t="n"/>
+      <c r="U73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4801,6 +4983,7 @@
       </c>
       <c r="S74" t="inlineStr"/>
       <c r="T74" s="2" t="n"/>
+      <c r="U74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4855,6 +5038,7 @@
       </c>
       <c r="S75" t="inlineStr"/>
       <c r="T75" s="2" t="n"/>
+      <c r="U75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4909,6 +5093,7 @@
       </c>
       <c r="S76" t="inlineStr"/>
       <c r="T76" s="2" t="n"/>
+      <c r="U76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4963,6 +5148,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" s="2" t="n"/>
+      <c r="U77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5017,6 +5203,7 @@
       </c>
       <c r="S78" t="inlineStr"/>
       <c r="T78" s="2" t="n"/>
+      <c r="U78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5071,6 +5258,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" s="2" t="n"/>
+      <c r="U79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5125,6 +5313,7 @@
       </c>
       <c r="S80" t="inlineStr"/>
       <c r="T80" s="2" t="n"/>
+      <c r="U80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5179,6 +5368,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" s="2" t="n"/>
+      <c r="U81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5233,6 +5423,7 @@
       </c>
       <c r="S82" t="inlineStr"/>
       <c r="T82" s="2" t="n"/>
+      <c r="U82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5287,6 +5478,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" s="2" t="n"/>
+      <c r="U83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5341,6 +5533,7 @@
       </c>
       <c r="S84" t="inlineStr"/>
       <c r="T84" s="2" t="n"/>
+      <c r="U84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5395,6 +5588,7 @@
       </c>
       <c r="S85" t="inlineStr"/>
       <c r="T85" s="2" t="n"/>
+      <c r="U85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5449,6 +5643,7 @@
       </c>
       <c r="S86" t="inlineStr"/>
       <c r="T86" s="2" t="n"/>
+      <c r="U86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5507,6 +5702,7 @@
         </is>
       </c>
       <c r="T87" s="2" t="n"/>
+      <c r="U87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5565,6 +5761,7 @@
         </is>
       </c>
       <c r="T88" s="2" t="n"/>
+      <c r="U88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5619,6 +5816,7 @@
       </c>
       <c r="S89" t="inlineStr"/>
       <c r="T89" s="2" t="n"/>
+      <c r="U89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5673,6 +5871,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" s="2" t="n"/>
+      <c r="U90" s="2" t="n"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5727,6 +5926,7 @@
       </c>
       <c r="S91" t="inlineStr"/>
       <c r="T91" s="2" t="n"/>
+      <c r="U91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5781,6 +5981,7 @@
       </c>
       <c r="S92" t="inlineStr"/>
       <c r="T92" s="2" t="n"/>
+      <c r="U92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5835,6 +6036,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" s="2" t="n"/>
+      <c r="U93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5889,6 +6091,7 @@
       </c>
       <c r="S94" t="inlineStr"/>
       <c r="T94" s="2" t="n"/>
+      <c r="U94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5943,6 +6146,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" s="2" t="n"/>
+      <c r="U95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5997,6 +6201,7 @@
       </c>
       <c r="S96" t="inlineStr"/>
       <c r="T96" s="2" t="n"/>
+      <c r="U96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6051,6 +6256,7 @@
       </c>
       <c r="S97" t="inlineStr"/>
       <c r="T97" s="2" t="n"/>
+      <c r="U97" s="2" t="n"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6105,6 +6311,7 @@
       </c>
       <c r="S98" t="inlineStr"/>
       <c r="T98" s="2" t="n"/>
+      <c r="U98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6159,6 +6366,7 @@
       </c>
       <c r="S99" t="inlineStr"/>
       <c r="T99" s="2" t="n"/>
+      <c r="U99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6213,6 +6421,7 @@
       </c>
       <c r="S100" t="inlineStr"/>
       <c r="T100" s="2" t="n"/>
+      <c r="U100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6267,6 +6476,7 @@
       </c>
       <c r="S101" t="inlineStr"/>
       <c r="T101" s="2" t="n"/>
+      <c r="U101" s="2" t="n"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6321,6 +6531,7 @@
       </c>
       <c r="S102" t="inlineStr"/>
       <c r="T102" s="2" t="n"/>
+      <c r="U102" s="2" t="n"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -6375,6 +6586,7 @@
       </c>
       <c r="S103" t="inlineStr"/>
       <c r="T103" s="2" t="n"/>
+      <c r="U103" s="2" t="n"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6429,6 +6641,7 @@
       </c>
       <c r="S104" t="inlineStr"/>
       <c r="T104" s="2" t="n"/>
+      <c r="U104" s="2" t="n"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -6483,6 +6696,7 @@
       </c>
       <c r="S105" t="inlineStr"/>
       <c r="T105" s="2" t="n"/>
+      <c r="U105" s="2" t="n"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -6534,6 +6748,7 @@
       <c r="Q106" t="inlineStr"/>
       <c r="S106" t="inlineStr"/>
       <c r="T106" s="2" t="n"/>
+      <c r="U106" s="2" t="n"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -6588,6 +6803,7 @@
       </c>
       <c r="S107" t="inlineStr"/>
       <c r="T107" s="2" t="n"/>
+      <c r="U107" s="2" t="n"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6642,6 +6858,7 @@
       </c>
       <c r="S108" t="inlineStr"/>
       <c r="T108" s="2" t="n"/>
+      <c r="U108" s="2" t="n"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6696,6 +6913,7 @@
       </c>
       <c r="S109" t="inlineStr"/>
       <c r="T109" s="2" t="n"/>
+      <c r="U109" s="2" t="n"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -6750,6 +6968,7 @@
       </c>
       <c r="S110" t="inlineStr"/>
       <c r="T110" s="2" t="n"/>
+      <c r="U110" s="2" t="n"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -6804,6 +7023,7 @@
       </c>
       <c r="S111" t="inlineStr"/>
       <c r="T111" s="2" t="n"/>
+      <c r="U111" s="2" t="n"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -6858,6 +7078,7 @@
       </c>
       <c r="S112" t="inlineStr"/>
       <c r="T112" s="2" t="n"/>
+      <c r="U112" s="2" t="n"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -6912,6 +7133,7 @@
       </c>
       <c r="S113" t="inlineStr"/>
       <c r="T113" s="2" t="n"/>
+      <c r="U113" s="2" t="n"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6966,6 +7188,7 @@
       </c>
       <c r="S114" t="inlineStr"/>
       <c r="T114" s="2" t="n"/>
+      <c r="U114" s="2" t="n"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -7020,6 +7243,7 @@
       </c>
       <c r="S115" t="inlineStr"/>
       <c r="T115" s="2" t="n"/>
+      <c r="U115" s="2" t="n"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -7074,6 +7298,7 @@
       </c>
       <c r="S116" t="inlineStr"/>
       <c r="T116" s="2" t="n"/>
+      <c r="U116" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7086,7 +7311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7228,6 +7453,21 @@
       <c r="C9" t="inlineStr">
         <is>
           <t>Para el precio mínimo (el piso).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Envío promedio que suma la competencia (USD)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Los precios de la calle no incluyen envío en tiendas especializadas (unos $7–15 bajo $50) y sí en Amazon/Walmart con Prime. Se promedian $5.</t>
         </is>
       </c>
     </row>
@@ -7286,7 +7526,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5. Precio de la calle: lo que he visto que cobran otras tiendas por el filtro original (capturas de búsqueda, pueden haber cambiado: verifícalos en Amazon, Walmart y Home Depot antes de publicar).</t>
+          <t>5. Calle puesta en la puerta: el precio que he visto en otras tiendas por el filtro original, más un envío promedio de $5 (las tiendas especializadas cobran envío; Amazon y Walmart con Prime no) (capturas de búsqueda, pueden haber cambiado: verifícalos en Amazon, Walmart y Home Depot antes de publicar).</t>
         </is>
       </c>
     </row>

</xml_diff>